<commit_message>
Refactor exposure rate handling and improve data loading in Fixed Radio Fluro components
- Enhanced API calls for fetching exposure rate data by implementing error handling and unwrapping response data for better usability.
- Updated the ExposureRateTableTop component to conditionally load data based on serviceId and testId, improving data management.
- Introduced a new utility function to handle data formatting and ensure consistent display of measurement values.
- Improved loading state management to provide better user feedback during data retrieval processes.
</commit_message>
<xml_diff>
--- a/public/templates/InterventionalRadiology_DoubleTube_Template.xlsx
+++ b/public/templates/InterventionalRadiology_DoubleTube_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:N119"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -745,368 +745,376 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>FDD (cm)</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B31" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C31" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D31" t="str">
-        <v>Time</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="F31" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="G31" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="H31" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="I31" t="str">
-        <v>Header 4</v>
-      </c>
-      <c r="J31" t="str">
-        <v>Header 5</v>
-      </c>
-      <c r="K31" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L31" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M31" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="N31" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O31" t="str">
-        <v>Meas 5</v>
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>100</v>
+        <v>Tolerance Sign</v>
       </c>
       <c r="B32" t="str">
-        <v>80</v>
-      </c>
-      <c r="C32" t="str">
-        <v>100</v>
-      </c>
-      <c r="D32" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="E32" t="str">
+        <v>&lt;=</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Tolerance Value (CoV)</v>
+      </c>
+      <c r="B33" t="str">
         <v>0.05</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Exposure 1</v>
-      </c>
-      <c r="G32" t="str">
-        <v>Exposure 2</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Exposure 3</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Exposure 4</v>
-      </c>
-      <c r="J32" t="str">
-        <v>Exposure 5</v>
-      </c>
-      <c r="K32" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="L32" t="str">
-        <v>0.51</v>
-      </c>
-      <c r="M32" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="N32" t="str">
-        <v>0.49</v>
-      </c>
-      <c r="O32" t="str">
-        <v>0.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION - Frontal</v>
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B34" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C34" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Time</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Header 4</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Header 5</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Meas 4</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Meas 5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Smallest Hole Size (mm)</v>
+        <v>100</v>
       </c>
       <c r="B35" t="str">
-        <v>Recommended Standard</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>1.0</v>
-      </c>
-      <c r="B36" t="str">
-        <v>&gt;= 1.0 mm</v>
+        <v>80</v>
+      </c>
+      <c r="C35" t="str">
+        <v>100</v>
+      </c>
+      <c r="D35" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Exposure 1</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Exposure 2</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Exposure 3</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Exposure 4</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Exposure 5</v>
+      </c>
+      <c r="J35" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="K35" t="str">
+        <v>0.51</v>
+      </c>
+      <c r="L35" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M35" t="str">
+        <v>0.49</v>
+      </c>
+      <c r="N35" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TEST: MEASUREMENT OF MA LINEARITY - Frontal</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION - Frontal</v>
+        <v>kVp</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Slice Thickness (mm)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Time (ms)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Tolerance</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="I38" t="str">
+        <v>mA Applied</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Meas 3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Measured Resolution (lp/mm)</v>
+        <v>80</v>
       </c>
       <c r="B39" t="str">
-        <v>Recommended Standard (lp/mm)</v>
+        <v>5</v>
+      </c>
+      <c r="C39" t="str">
+        <v>100</v>
+      </c>
+      <c r="D39" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="E39" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="I39" t="str">
+        <v>50</v>
+      </c>
+      <c r="J39" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="K39" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="L39" t="str">
+        <v>0.09</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2.0</v>
+        <v/>
       </c>
       <c r="B40" t="str">
-        <v>&gt;= 2.0 lp/mm</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP - Frontal</v>
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v>100</v>
+      </c>
+      <c r="J40" t="str">
+        <v>0.20</v>
+      </c>
+      <c r="K40" t="str">
+        <v>0.21</v>
+      </c>
+      <c r="L40" t="str">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v>200</v>
+      </c>
+      <c r="J41" t="str">
+        <v>0.40</v>
+      </c>
+      <c r="K41" t="str">
+        <v>0.41</v>
+      </c>
+      <c r="L41" t="str">
+        <v>0.39</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
-      </c>
-      <c r="B43" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
-      </c>
-      <c r="C43" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Distance (cm)</v>
-      </c>
-      <c r="E43" t="str">
-        <v>kV</v>
-      </c>
-      <c r="F43" t="str">
-        <v>mA</v>
-      </c>
-      <c r="G43" t="str">
-        <v>Mode</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Measured Rate</v>
-      </c>
-      <c r="I43" t="str">
-        <v>Criteria</v>
+        <v>TEST: LOW CONTRAST RESOLUTION - Frontal</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>10</v>
+        <v>Smallest Hole Size (mm)</v>
       </c>
       <c r="B44" t="str">
-        <v>5</v>
-      </c>
-      <c r="C44" t="str">
-        <v>30</v>
-      </c>
-      <c r="D44" t="str">
-        <v>100</v>
-      </c>
-      <c r="E44" t="str">
-        <v>80</v>
-      </c>
-      <c r="F44" t="str">
-        <v>100</v>
-      </c>
-      <c r="G44" t="str">
-        <v>AEC</v>
-      </c>
-      <c r="H44" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="I44" t="str">
-        <v>5</v>
+        <v>Recommended Standard</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="B45" t="str">
-        <v/>
-      </c>
-      <c r="C45" t="str">
-        <v/>
-      </c>
-      <c r="D45" t="str">
-        <v>100</v>
-      </c>
-      <c r="E45" t="str">
-        <v>80</v>
-      </c>
-      <c r="F45" t="str">
-        <v>100</v>
-      </c>
-      <c r="G45" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="H45" t="str">
-        <v>2.5</v>
-      </c>
-      <c r="I45" t="str">
-        <v>5</v>
+        <v>&gt;= 1.0 mm</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE - Frontal</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION - Frontal</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>kV</v>
+        <v>Measured Resolution (lp/mm)</v>
       </c>
       <c r="B48" t="str">
-        <v>mA</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Time</v>
-      </c>
-      <c r="D48" t="str">
-        <v>FDD (cm)</v>
-      </c>
-      <c r="E48" t="str">
-        <v>Workload</v>
-      </c>
-      <c r="F48" t="str">
-        <v>Location</v>
-      </c>
-      <c r="G48" t="str">
-        <v>Left</v>
-      </c>
-      <c r="H48" t="str">
-        <v>Right</v>
-      </c>
-      <c r="I48" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J48" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K48" t="str">
-        <v>Top</v>
-      </c>
-      <c r="L48" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="M48" t="str">
-        <v>Tolerance Value</v>
+        <v>Recommended Standard (lp/mm)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>120</v>
+        <v>2.0</v>
       </c>
       <c r="B49" t="str">
-        <v>21</v>
-      </c>
-      <c r="C49" t="str">
-        <v>2</v>
-      </c>
-      <c r="D49" t="str">
-        <v>100</v>
-      </c>
-      <c r="E49" t="str">
-        <v>5000</v>
-      </c>
-      <c r="F49" t="str">
-        <v>Tube</v>
-      </c>
-      <c r="G49" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="H49" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="I49" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="J49" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="K49" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="L49" t="str">
-        <v>&lt;=</v>
-      </c>
-      <c r="M49" t="str">
-        <v>1</v>
+        <v>&gt;= 2.0 lp/mm</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>TEST: ACCURACY OF IRRADIATION TIME - Lateral</v>
+        <v>TEST: EXPOSURE RATE AT TABLE TOP - Frontal</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>FDD (cm)</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
       </c>
       <c r="B52" t="str">
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Min. Focus to Tabletop Distance</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Distance (cm)</v>
+      </c>
+      <c r="E52" t="str">
         <v>kV</v>
       </c>
-      <c r="C52" t="str">
+      <c r="F52" t="str">
         <v>mA</v>
       </c>
-      <c r="D52" t="str">
-        <v>Set Time (mSec)</v>
-      </c>
-      <c r="E52" t="str">
-        <v>Measured Time (mSec)</v>
-      </c>
-      <c r="F52" t="str">
-        <v>Tolerance Operator</v>
-      </c>
       <c r="G52" t="str">
-        <v>Tolerance Value</v>
+        <v>Mode</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Measured Rate</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Criteria</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="B53" t="str">
+        <v>5</v>
+      </c>
+      <c r="C53" t="str">
+        <v>30</v>
+      </c>
+      <c r="D53" t="str">
+        <v>100</v>
+      </c>
+      <c r="E53" t="str">
         <v>80</v>
       </c>
-      <c r="C53" t="str">
-        <v>100</v>
-      </c>
-      <c r="D53" t="str">
-        <v>200</v>
-      </c>
-      <c r="E53" t="str">
-        <v>198</v>
-      </c>
       <c r="F53" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
       </c>
       <c r="G53" t="str">
-        <v>10</v>
+        <v>AEC</v>
+      </c>
+      <c r="H53" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="I53" t="str">
+        <v>5</v>
       </c>
     </row>
     <row r="54">
@@ -1120,318 +1128,324 @@
         <v/>
       </c>
       <c r="D54" t="str">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="E54" t="str">
-        <v>497</v>
+        <v>80</v>
       </c>
       <c r="F54" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
       </c>
       <c r="G54" t="str">
-        <v>10</v>
+        <v>Manual</v>
+      </c>
+      <c r="H54" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I54" t="str">
+        <v>5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>TEST: CENTRAL BEAM ALIGNMENT - Lateral</v>
+        <v>TEST: TUBE HOUSING LEAKAGE - Frontal</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>FFD (cm)</v>
+        <v>kV</v>
       </c>
       <c r="B57" t="str">
-        <v>100</v>
+        <v>mA</v>
       </c>
       <c r="C57" t="str">
-        <v>kV</v>
+        <v>Time</v>
       </c>
       <c r="D57" t="str">
-        <v>80</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="E57" t="str">
-        <v>mA</v>
+        <v>Workload</v>
       </c>
       <c r="F57" t="str">
-        <v>100</v>
+        <v>Location</v>
       </c>
       <c r="G57" t="str">
-        <v>Time</v>
+        <v>Left</v>
       </c>
       <c r="H57" t="str">
-        <v>0.1</v>
+        <v>Right</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Front</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Back</v>
+      </c>
+      <c r="K57" t="str">
+        <v>Top</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Tolerance Value</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Observed Tilt (cm)</v>
+        <v>120</v>
       </c>
       <c r="B58" t="str">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="B59" t="str">
+        <v>21</v>
+      </c>
+      <c r="C58" t="str">
+        <v>2</v>
+      </c>
+      <c r="D58" t="str">
+        <v>100</v>
+      </c>
+      <c r="E58" t="str">
+        <v>5000</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="G58" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="H58" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="I58" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="J58" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="K58" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="L58" t="str">
         <v>&lt;=</v>
+      </c>
+      <c r="M58" t="str">
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Tolerance Value (cm)</v>
-      </c>
-      <c r="B60" t="str">
-        <v>1.5</v>
+        <v>TEST: ACCURACY OF IRRADIATION TIME - Lateral</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B61" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C61" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Set Time (mSec)</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Measured Time (mSec)</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Tolerance Value</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>TEST: EFFECTIVE FOCAL SPOT SIZE - Lateral</v>
+        <v>100</v>
+      </c>
+      <c r="B62" t="str">
+        <v>80</v>
+      </c>
+      <c r="C62" t="str">
+        <v>100</v>
+      </c>
+      <c r="D62" t="str">
+        <v>200</v>
+      </c>
+      <c r="E62" t="str">
+        <v>198</v>
+      </c>
+      <c r="F62" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="G62" t="str">
+        <v>10</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>FFD (cm)</v>
+        <v/>
       </c>
       <c r="B63" t="str">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>Focus Type</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Stated Focal Spot (mm)</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Measured Focal Spot (Nominal) (mm)</v>
+        <v/>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63" t="str">
+        <v>500</v>
+      </c>
+      <c r="E63" t="str">
+        <v>497</v>
+      </c>
+      <c r="F63" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="G63" t="str">
+        <v>10</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Large Focus</v>
-      </c>
-      <c r="B65" t="str">
-        <v>2</v>
-      </c>
-      <c r="C65" t="str">
-        <v>1.25</v>
+        <v>TEST: CENTRAL BEAM ALIGNMENT - Lateral</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Small Focus</v>
+        <v>FFD (cm)</v>
       </c>
       <c r="B66" t="str">
-        <v>0.6</v>
+        <v>100</v>
       </c>
       <c r="C66" t="str">
-        <v>0.65</v>
+        <v>kV</v>
+      </c>
+      <c r="D66" t="str">
+        <v>80</v>
+      </c>
+      <c r="E66" t="str">
+        <v>mA</v>
+      </c>
+      <c r="F66" t="str">
+        <v>100</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Time</v>
+      </c>
+      <c r="H66" t="str">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Observed Tilt (cm)</v>
+      </c>
+      <c r="B67" t="str">
+        <v>0.5</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>TEST: ACCURACY OF OPERATING POTENTIAL - Lateral</v>
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B68" t="str">
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>mA</v>
+        <v>Tolerance Value (cm)</v>
       </c>
       <c r="B69" t="str">
-        <v>Time</v>
-      </c>
-      <c r="C69" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="D69" t="str">
-        <v>Tolerance Value</v>
-      </c>
-      <c r="E69" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="F69" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="G69" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="H69" t="str">
-        <v>Set kV</v>
-      </c>
-      <c r="I69" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="J69" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K69" t="str">
-        <v>Meas 3</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v>100</v>
-      </c>
-      <c r="B70" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="C70" t="str">
-        <v>&lt;=</v>
-      </c>
-      <c r="D70" t="str">
-        <v>5</v>
-      </c>
-      <c r="E70" t="str">
-        <v>50 mA</v>
-      </c>
-      <c r="F70" t="str">
-        <v>100 mA</v>
-      </c>
-      <c r="G70" t="str">
-        <v>200 mA</v>
-      </c>
-      <c r="H70" t="str">
-        <v>60</v>
-      </c>
-      <c r="I70" t="str">
-        <v>59.8</v>
-      </c>
-      <c r="J70" t="str">
-        <v>60.2</v>
-      </c>
-      <c r="K70" t="str">
-        <v>60</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v/>
-      </c>
-      <c r="B71" t="str">
-        <v/>
-      </c>
-      <c r="C71" t="str">
-        <v/>
-      </c>
-      <c r="D71" t="str">
-        <v/>
-      </c>
-      <c r="E71" t="str">
-        <v/>
-      </c>
-      <c r="F71" t="str">
-        <v/>
-      </c>
-      <c r="G71" t="str">
-        <v/>
-      </c>
-      <c r="H71" t="str">
-        <v>80</v>
-      </c>
-      <c r="I71" t="str">
-        <v>79.8</v>
-      </c>
-      <c r="J71" t="str">
-        <v>80.1</v>
-      </c>
-      <c r="K71" t="str">
-        <v>79.9</v>
+        <v>TEST: EFFECTIVE FOCAL SPOT SIZE - Lateral</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>FFD (cm)</v>
+      </c>
+      <c r="B72" t="str">
+        <v>100</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>TEST: TOTAL FILTRATION - Lateral</v>
+        <v>Focus Type</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Stated Focal Spot (mm)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Measured Focal Spot (Nominal) (mm)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Applied KV</v>
+        <v>Large Focus</v>
       </c>
       <c r="B74" t="str">
-        <v>Applied MA</v>
+        <v>2</v>
       </c>
       <c r="C74" t="str">
-        <v>Applied Time</v>
-      </c>
-      <c r="D74" t="str">
-        <v>Measured TF</v>
-      </c>
-      <c r="E74" t="str">
-        <v>Criteria</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>80</v>
+        <v>Small Focus</v>
       </c>
       <c r="B75" t="str">
-        <v>100</v>
+        <v>0.6</v>
       </c>
       <c r="C75" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="D75" t="str">
-        <v>2.6</v>
-      </c>
-      <c r="E75" t="str">
-        <v>2.5</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>TEST: CONSISTENCY OF RADIATION OUTPUT - Lateral</v>
+        <v>TEST: ACCURACY OF OPERATING POTENTIAL - Lateral</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>FDD (cm)</v>
+        <v>mA</v>
       </c>
       <c r="B78" t="str">
-        <v>kV</v>
+        <v>Time</v>
       </c>
       <c r="C78" t="str">
-        <v>mA</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="D78" t="str">
-        <v>Time</v>
+        <v>Tolerance Value</v>
       </c>
       <c r="E78" t="str">
-        <v>Tolerance</v>
+        <v>Header 1</v>
       </c>
       <c r="F78" t="str">
-        <v>Header 1</v>
+        <v>Header 2</v>
       </c>
       <c r="G78" t="str">
-        <v>Header 2</v>
+        <v>Header 3</v>
       </c>
       <c r="H78" t="str">
-        <v>Header 3</v>
+        <v>Set kV</v>
       </c>
       <c r="I78" t="str">
-        <v>Header 4</v>
+        <v>Meas 1</v>
       </c>
       <c r="J78" t="str">
-        <v>Header 5</v>
+        <v>Meas 2</v>
       </c>
       <c r="K78" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L78" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M78" t="str">
         <v>Meas 3</v>
-      </c>
-      <c r="N78" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O78" t="str">
-        <v>Meas 5</v>
       </c>
     </row>
     <row r="79">
@@ -1439,346 +1453,682 @@
         <v>100</v>
       </c>
       <c r="B79" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="C79" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="D79" t="str">
+        <v>5</v>
+      </c>
+      <c r="E79" t="str">
+        <v>50 mA</v>
+      </c>
+      <c r="F79" t="str">
+        <v>100 mA</v>
+      </c>
+      <c r="G79" t="str">
+        <v>200 mA</v>
+      </c>
+      <c r="H79" t="str">
+        <v>60</v>
+      </c>
+      <c r="I79" t="str">
+        <v>59.8</v>
+      </c>
+      <c r="J79" t="str">
+        <v>60.2</v>
+      </c>
+      <c r="K79" t="str">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v/>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
         <v>80</v>
       </c>
-      <c r="C79" t="str">
-        <v>100</v>
-      </c>
-      <c r="D79" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="E79" t="str">
-        <v>0.05</v>
-      </c>
-      <c r="F79" t="str">
-        <v>Exposure 1</v>
-      </c>
-      <c r="G79" t="str">
-        <v>Exposure 2</v>
-      </c>
-      <c r="H79" t="str">
-        <v>Exposure 3</v>
-      </c>
-      <c r="I79" t="str">
-        <v>Exposure 4</v>
-      </c>
-      <c r="J79" t="str">
-        <v>Exposure 5</v>
-      </c>
-      <c r="K79" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="L79" t="str">
-        <v>0.51</v>
-      </c>
-      <c r="M79" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="N79" t="str">
-        <v>0.49</v>
-      </c>
-      <c r="O79" t="str">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION - Lateral</v>
+      <c r="I80" t="str">
+        <v>79.8</v>
+      </c>
+      <c r="J80" t="str">
+        <v>80.1</v>
+      </c>
+      <c r="K80" t="str">
+        <v>79.9</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Smallest Hole Size (mm)</v>
-      </c>
-      <c r="B82" t="str">
-        <v>Recommended Standard</v>
+        <v>TEST: TOTAL FILTRATION - Lateral</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>1.0</v>
+        <v>Applied KV</v>
       </c>
       <c r="B83" t="str">
-        <v>&gt;= 1.0 mm</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION - Lateral</v>
+        <v>Applied MA</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Applied Time</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Measured TF</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Criteria</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>80</v>
+      </c>
+      <c r="B84" t="str">
+        <v>100</v>
+      </c>
+      <c r="C84" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="D84" t="str">
+        <v>2.6</v>
+      </c>
+      <c r="E84" t="str">
+        <v>2.5</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Measured Resolution (lp/mm)</v>
-      </c>
-      <c r="B86" t="str">
-        <v>Recommended Standard (lp/mm)</v>
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT - Lateral</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2.0</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B87" t="str">
-        <v>&gt;= 2.0 lp/mm</v>
+        <v>&lt;=</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Tolerance Sign</v>
+      </c>
+      <c r="B88" t="str">
+        <v>&lt;=</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP - Lateral</v>
+        <v>Tolerance Value (CoV)</v>
+      </c>
+      <c r="B89" t="str">
+        <v>0.05</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B90" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+        <v>kV</v>
       </c>
       <c r="C90" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
+        <v>mA</v>
       </c>
       <c r="D90" t="str">
-        <v>Distance (cm)</v>
+        <v>Time</v>
       </c>
       <c r="E90" t="str">
-        <v>kV</v>
+        <v>Header 1</v>
       </c>
       <c r="F90" t="str">
-        <v>mA</v>
+        <v>Header 2</v>
       </c>
       <c r="G90" t="str">
-        <v>Mode</v>
+        <v>Header 3</v>
       </c>
       <c r="H90" t="str">
-        <v>Measured Rate</v>
+        <v>Header 4</v>
       </c>
       <c r="I90" t="str">
-        <v>Criteria</v>
+        <v>Header 5</v>
+      </c>
+      <c r="J90" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="K90" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="L90" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="M90" t="str">
+        <v>Meas 4</v>
+      </c>
+      <c r="N90" t="str">
+        <v>Meas 5</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B91" t="str">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="C91" t="str">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D91" t="str">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E91" t="str">
-        <v>80</v>
+        <v>Exposure 1</v>
       </c>
       <c r="F91" t="str">
-        <v>100</v>
+        <v>Exposure 2</v>
       </c>
       <c r="G91" t="str">
-        <v>AEC</v>
+        <v>Exposure 3</v>
       </c>
       <c r="H91" t="str">
+        <v>Exposure 4</v>
+      </c>
+      <c r="I91" t="str">
+        <v>Exposure 5</v>
+      </c>
+      <c r="J91" t="str">
         <v>0.5</v>
       </c>
-      <c r="I91" t="str">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="str">
-        <v/>
-      </c>
-      <c r="B92" t="str">
-        <v/>
-      </c>
-      <c r="C92" t="str">
-        <v/>
-      </c>
-      <c r="D92" t="str">
-        <v>100</v>
-      </c>
-      <c r="E92" t="str">
-        <v>80</v>
-      </c>
-      <c r="F92" t="str">
-        <v>100</v>
-      </c>
-      <c r="G92" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="H92" t="str">
-        <v>2.5</v>
-      </c>
-      <c r="I92" t="str">
-        <v>5</v>
+      <c r="K91" t="str">
+        <v>0.51</v>
+      </c>
+      <c r="L91" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="M91" t="str">
+        <v>0.49</v>
+      </c>
+      <c r="N91" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>TEST: MEASUREMENT OF MA LINEARITY - Lateral</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE - Lateral</v>
+        <v>kVp</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Slice Thickness (mm)</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Time (ms)</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Tolerance</v>
+      </c>
+      <c r="F94" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="H94" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="I94" t="str">
+        <v>mA Applied</v>
+      </c>
+      <c r="J94" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="K94" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="L94" t="str">
+        <v>Meas 3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>kV</v>
+        <v>80</v>
       </c>
       <c r="B95" t="str">
-        <v>mA</v>
+        <v>5</v>
       </c>
       <c r="C95" t="str">
-        <v>Time</v>
+        <v>100</v>
       </c>
       <c r="D95" t="str">
-        <v>FDD (cm)</v>
+        <v>&lt;=</v>
       </c>
       <c r="E95" t="str">
-        <v>Workload</v>
+        <v>0.1</v>
       </c>
       <c r="F95" t="str">
-        <v>Location</v>
+        <v>Meas 1</v>
       </c>
       <c r="G95" t="str">
-        <v>Left</v>
+        <v>Meas 2</v>
       </c>
       <c r="H95" t="str">
-        <v>Right</v>
+        <v>Meas 3</v>
       </c>
       <c r="I95" t="str">
-        <v>Front</v>
+        <v>50</v>
       </c>
       <c r="J95" t="str">
-        <v>Back</v>
+        <v>0.10</v>
       </c>
       <c r="K95" t="str">
-        <v>Top</v>
+        <v>0.11</v>
       </c>
       <c r="L95" t="str">
-        <v>Tolerance Operator</v>
-      </c>
-      <c r="M95" t="str">
-        <v>Tolerance Value</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>120</v>
+        <v/>
       </c>
       <c r="B96" t="str">
-        <v>21</v>
+        <v/>
       </c>
       <c r="C96" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="D96" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="E96" t="str">
-        <v>5000</v>
+        <v/>
       </c>
       <c r="F96" t="str">
-        <v>Tube</v>
+        <v/>
       </c>
       <c r="G96" t="str">
-        <v>0.1</v>
+        <v/>
       </c>
       <c r="H96" t="str">
-        <v>0.1</v>
+        <v/>
       </c>
       <c r="I96" t="str">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="J96" t="str">
-        <v>0.1</v>
+        <v>0.20</v>
       </c>
       <c r="K96" t="str">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="L96" t="str">
-        <v>&lt;=</v>
-      </c>
-      <c r="M96" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v/>
+      </c>
+      <c r="B97" t="str">
+        <v/>
+      </c>
+      <c r="C97" t="str">
+        <v/>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v/>
+      </c>
+      <c r="G97" t="str">
+        <v/>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v>200</v>
+      </c>
+      <c r="J97" t="str">
+        <v>0.40</v>
+      </c>
+      <c r="K97" t="str">
+        <v>0.41</v>
+      </c>
+      <c r="L97" t="str">
+        <v>0.39</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Location</v>
-      </c>
-      <c r="B99" t="str">
-        <v>mR/hr</v>
-      </c>
-      <c r="C99" t="str">
-        <v>Category</v>
-      </c>
-      <c r="D99" t="str">
-        <v>Applied Voltage</v>
-      </c>
-      <c r="E99" t="str">
-        <v>Applied Current</v>
-      </c>
-      <c r="F99" t="str">
-        <v>Exposure Time</v>
-      </c>
-      <c r="G99" t="str">
-        <v>Workload</v>
+        <v>TEST: LOW CONTRAST RESOLUTION - Lateral</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Control Console</v>
+        <v>Smallest Hole Size (mm)</v>
       </c>
       <c r="B100" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="C100" t="str">
-        <v>worker</v>
-      </c>
-      <c r="D100" t="str">
-        <v>80</v>
-      </c>
-      <c r="E100" t="str">
-        <v>100</v>
-      </c>
-      <c r="F100" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="G100" t="str">
-        <v>5000</v>
+        <v>Recommended Standard</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="B101" t="str">
+        <v>&gt;= 1.0 mm</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>TEST: HIGH CONTRAST RESOLUTION - Lateral</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Recommended Standard (lp/mm)</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2.0</v>
+      </c>
+      <c r="B105" t="str">
+        <v>&gt;= 2.0 lp/mm</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>TEST: EXPOSURE RATE AT TABLE TOP - Lateral</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Min. Focus to Tabletop Distance</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Distance (cm)</v>
+      </c>
+      <c r="E108" t="str">
+        <v>kV</v>
+      </c>
+      <c r="F108" t="str">
+        <v>mA</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Mode</v>
+      </c>
+      <c r="H108" t="str">
+        <v>Measured Rate</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Criteria</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>10</v>
+      </c>
+      <c r="B109" t="str">
+        <v>5</v>
+      </c>
+      <c r="C109" t="str">
+        <v>30</v>
+      </c>
+      <c r="D109" t="str">
+        <v>100</v>
+      </c>
+      <c r="E109" t="str">
+        <v>80</v>
+      </c>
+      <c r="F109" t="str">
+        <v>100</v>
+      </c>
+      <c r="G109" t="str">
+        <v>AEC</v>
+      </c>
+      <c r="H109" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="I109" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v/>
+      </c>
+      <c r="B110" t="str">
+        <v/>
+      </c>
+      <c r="C110" t="str">
+        <v/>
+      </c>
+      <c r="D110" t="str">
+        <v>100</v>
+      </c>
+      <c r="E110" t="str">
+        <v>80</v>
+      </c>
+      <c r="F110" t="str">
+        <v>100</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="H110" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I110" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>TEST: TUBE HOUSING LEAKAGE - Lateral</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>kV</v>
+      </c>
+      <c r="B113" t="str">
+        <v>mA</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Time</v>
+      </c>
+      <c r="D113" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Workload</v>
+      </c>
+      <c r="F113" t="str">
+        <v>Location</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Left</v>
+      </c>
+      <c r="H113" t="str">
+        <v>Right</v>
+      </c>
+      <c r="I113" t="str">
+        <v>Front</v>
+      </c>
+      <c r="J113" t="str">
+        <v>Back</v>
+      </c>
+      <c r="K113" t="str">
+        <v>Top</v>
+      </c>
+      <c r="L113" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="M113" t="str">
+        <v>Tolerance Value</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>120</v>
+      </c>
+      <c r="B114" t="str">
+        <v>21</v>
+      </c>
+      <c r="C114" t="str">
+        <v>2</v>
+      </c>
+      <c r="D114" t="str">
+        <v>100</v>
+      </c>
+      <c r="E114" t="str">
+        <v>5000</v>
+      </c>
+      <c r="F114" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="G114" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="H114" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="I114" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="J114" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="K114" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="L114" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="M114" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>TEST: RADIATION PROTECTION SURVEY REPORT</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Location</v>
+      </c>
+      <c r="B117" t="str">
+        <v>mR/hr</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Applied Voltage</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Applied Current</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Exposure Time</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Workload</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Control Console</v>
+      </c>
+      <c r="B118" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="C118" t="str">
+        <v>worker</v>
+      </c>
+      <c r="D118" t="str">
+        <v>80</v>
+      </c>
+      <c r="E118" t="str">
+        <v>100</v>
+      </c>
+      <c r="F118" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="G118" t="str">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
         <v>Entrance Door</v>
       </c>
-      <c r="B101" t="str">
+      <c r="B119" t="str">
         <v>0.05</v>
       </c>
-      <c r="C101" t="str">
+      <c r="C119" t="str">
         <v>public</v>
       </c>
-      <c r="D101" t="str">
-        <v/>
-      </c>
-      <c r="E101" t="str">
-        <v/>
-      </c>
-      <c r="F101" t="str">
-        <v/>
-      </c>
-      <c r="G101" t="str">
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119" t="str">
+        <v/>
+      </c>
+      <c r="G119" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N119"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>